<commit_message>
Refactor Excel file import logic to handle null cells and improve plan data extraction; update main method to display imported plans
</commit_message>
<xml_diff>
--- a/.excel/plans.xlsx
+++ b/.excel/plans.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/one/IdeaProjects/cpiForecast/.excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{203BA888-4F08-E140-81C1-1A9F66FF8002}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8AAEBC-F2C4-B047-8076-1170E005D91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5040" yWindow="1800" windowWidth="28300" windowHeight="17440" xr2:uid="{668DB8E8-A5D0-1E48-999F-BD4BCE261E1C}"/>
+    <workbookView xWindow="5040" yWindow="1800" windowWidth="28300" windowHeight="17440" activeTab="1" xr2:uid="{668DB8E8-A5D0-1E48-999F-BD4BCE261E1C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="サンプル" sheetId="1" r:id="rId1"/>
+    <sheet name="9月" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,8 +35,39 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>one</author>
+  </authors>
+  <commentList>
+    <comment ref="Z5" authorId="0" shapeId="0" xr:uid="{91A66D6A-E72B-D34A-B3CD-3BD9AB0F80D9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Yu Gothic UI"/>
+          </rPr>
+          <t>one:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color rgb="FF000000"/>
+            <rFont val="Yu Gothic UI"/>
+          </rPr>
+          <t>この列に値がはいっていないとリストにいれない</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="4">
   <si>
     <t>改修プラン1(CPI1以上のサンプル)</t>
     <rPh sb="0" eb="2">
@@ -60,7 +92,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -75,6 +107,17 @@
       <family val="2"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Yu Gothic UI"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Yu Gothic UI"/>
     </font>
   </fonts>
   <fills count="2">
@@ -469,4 +512,61 @@
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3C7471A-AD14-534D-87BE-7C7207639C1A}">
+  <dimension ref="B5:Z7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="20"/>
+  <cols>
+    <col min="4" max="4" width="30" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="2:26">
+      <c r="B5">
+        <v>123</v>
+      </c>
+      <c r="D5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="2:26">
+      <c r="B6">
+        <v>456</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z6">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="2:26">
+      <c r="B7">
+        <v>789</v>
+      </c>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1</v>
+      </c>
+      <c r="Z7">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>